<commit_message>
Updated NZL_grids model - 2025-09-07 16:38
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF98D378-E54E-4CE0-97F8-6434A4C98C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{88C15B4A-E029-4363-851D-B59C0ED84FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5441,7 +5441,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1969FC93-564F-400B-9296-322EAA3B637A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC27DBB9-71BD-4FC0-A1C8-74CEC9F698D4}">
   <dimension ref="B9:D248"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8085,7 +8085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82F6B4BF-D58F-4707-A11C-D47627FC370F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{989AF825-AC80-4291-85AC-2D58401542FE}">
   <dimension ref="B2:D241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-07 23:22
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BFCE000-0303-44FE-87B3-D810783A4595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B4B62D63-C964-45E3-8BC0-EA297242A488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6725,7 +6725,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ED6EA9C-3E4C-4261-AC3F-0EAB516749D8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E68F0C6A-3DDE-4C92-BBC2-852BC788A30A}">
   <dimension ref="B9:D676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14077,7 +14077,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BD4E5D4-00B2-48E6-AD1B-69B8B98A90BE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49EFACAD-9B55-44F5-9B7F-AF5F2C4A0216}">
   <dimension ref="B2:D669"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-09 11:31
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FCE6C87-D8C9-4D93-8ADF-A0AD29051DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{159DAB07-CADD-4F9C-A09C-6972AC2B5D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9129,7 +9129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8191D3E7-570D-4EF7-8FD1-42D7F5B3DFC2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85168240-2819-412C-81E8-5895D18F50A4}">
   <dimension ref="B9:D676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -16481,7 +16481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8EDAB4F-EA3A-461C-A84D-991CDA6B1EB1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80139961-872B-4A33-8A9E-1A0226222230}">
   <dimension ref="B9:H676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-09 21:20
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{159DAB07-CADD-4F9C-A09C-6972AC2B5D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8778596A-AE0B-4451-9C18-88D63EDB7EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9129,7 +9129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85168240-2819-412C-81E8-5895D18F50A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4AB9B60-92D3-4739-8631-8DE66F4A9F84}">
   <dimension ref="B9:D676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -16481,7 +16481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80139961-872B-4A33-8A9E-1A0226222230}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2851D56E-9638-45F1-9DC5-D1A045FF774F}">
   <dimension ref="B9:H676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-09 23:33
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8778596A-AE0B-4451-9C18-88D63EDB7EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14ED6E37-8F7A-4B24-A4C8-FC7647EB1802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9129,7 +9129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4AB9B60-92D3-4739-8631-8DE66F4A9F84}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D639A65-2009-40C0-AD67-C65139818F53}">
   <dimension ref="B9:D676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -16481,7 +16481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2851D56E-9638-45F1-9DC5-D1A045FF774F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1257A1-917F-4789-8579-489D597A82F6}">
   <dimension ref="B9:H676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-17 02:47
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07FF8FD8-EECA-4CFC-8FB5-67C4BADDAD32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCE063CB-F4A1-4AE8-86B8-0FADD9A6ECD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="12683" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -1241,13 +1241,13 @@
     <t>g64</t>
   </si>
   <si>
-    <t>f97p50</t>
-  </si>
-  <si>
     <t>f96p10</t>
   </si>
   <si>
     <t>f96p90</t>
+  </si>
+  <si>
+    <t>f96p50</t>
   </si>
   <si>
     <t>grid_node</t>
@@ -7052,7 +7052,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D921485-FD48-41A0-9773-A9C096BA364A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A602EE4-BFE0-44DA-8D50-447105598C8E}">
   <dimension ref="B9:D676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14404,7 +14404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2AFF8E6-5445-42F2-A557-FB4F3086F9C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B8236BF-C490-44B1-BFFC-A0957FBF8177}">
   <dimension ref="B9:H676"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28195,7 +28195,7 @@
         <v>337</v>
       </c>
       <c r="U12" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" spans="2:24">
@@ -28238,7 +28238,7 @@
         <v>343</v>
       </c>
       <c r="U13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="14" spans="2:24">
@@ -28281,7 +28281,7 @@
         <v>349</v>
       </c>
       <c r="U14" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="2:24">
@@ -29098,11 +29098,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -29110,7 +29110,7 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N36">
         <v>5</v>
@@ -29135,11 +29135,11 @@
       </c>
       <c r="C37" t="str">
         <f t="shared" si="5"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="3"/>
@@ -29147,7 +29147,7 @@
       </c>
       <c r="J37" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N37">
         <v>5</v>
@@ -29172,11 +29172,11 @@
       </c>
       <c r="C38" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="3"/>
@@ -29184,7 +29184,7 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N38">
         <v>5</v>
@@ -29209,11 +29209,11 @@
       </c>
       <c r="C39" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="I39" t="str">
         <f t="shared" si="3"/>
@@ -29221,7 +29221,7 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N39">
         <v>5</v>
@@ -29246,11 +29246,11 @@
       </c>
       <c r="C40" t="str">
         <f t="shared" si="5"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="I40" t="str">
         <f t="shared" si="3"/>
@@ -29258,7 +29258,7 @@
       </c>
       <c r="J40" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N40">
         <v>5</v>

</xml_diff>